<commit_message>
BSI.IT.27.C7: limit final package strictly to period 07/2025-06/2026
- Remove 2026 Q2 (after period) from walkthrough, WP2 and Sample of 1
- Exceptions now 16 accounts (in-period only); results unchanged
- Drop subsequent-period folder; Q2_2026 workbook kept outside the final folder
- Index updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GtAt3iBzX5VYFEMTgXwPkP
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7 Network Device Admin Accoun/BSI.IT.27.C7 Final 07.2025-06.2026/BSI.IT.27.C7 Final Package Index.xlsx
+++ b/BSI.IT.27.C7 Network Device Admin Accoun/BSI.IT.27.C7 Final 07.2025-06.2026/BSI.IT.27.C7 Final Package Index.xlsx
@@ -73,16 +73,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -450,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -471,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Testing period: 07/01/2025 - 06/30/2026  |  Conclusion: Needs Improvement (Sample 1 2025 Q3 FAIL A5/A6; Sample 2 2026 Q1 FAIL A5)</t>
+          <t>Testing period: 07/01/2025 - 06/30/2026 (July 2025 - June 2026)  |  Conclusion: Needs Improvement - Sample 1 2025 Q3 FAIL (A5, A6); Sample 2 2026 Q1 FAIL (A5)</t>
         </is>
       </c>
     </row>
@@ -532,15 +529,15 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Sample of 1 - 2026 Q1 certification walkthrough with exhibits</t>
+          <t>Sample of 1 - 2026 Q1 certification with exhibits</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
-        <v>1647</v>
+        <v>1637</v>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>45ef576cd6602e0b89059e820e43301a</t>
+          <t>5188edcf64c89013aa3e8b8ba984ef06</t>
         </is>
       </c>
     </row>
@@ -562,15 +559,15 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Step-by-step testing, attribute matrix A1-A7, exceptions, sources, evidence status</t>
+          <t>Step-by-step testing, attribute matrix A1-A7, item detail, exceptions (16 accounts), sources, evidence status</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>b666da3432931a6a25e7763154f117d9</t>
+          <t>880b5baa061deffdede0a55e52cb9a8b</t>
         </is>
       </c>
     </row>
@@ -592,7 +589,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Control Metadata, CDA, CPA (samples 2025 Q3 and 2026 Q1, rating)</t>
+          <t>Control Metadata, CDA, CPA (samples 2025 Q3 and 2026 Q1, rating Needs Improvement)</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -600,7 +597,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>37cd30a101f16d136b61ed90881ef3fd</t>
+          <t>80008be6086194f4129cc4f963d43874</t>
         </is>
       </c>
     </row>
@@ -707,12 +704,12 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>In period - SAMPLE 2 (H1 2026)</t>
+          <t>SAMPLE 2 - covers Jan-Jun 2026</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>2026 Q1 SOX certification (launched 4/9/2026), AD extract 05/15/2026, Netwrix revocations</t>
+          <t>2026 Q1 SOX certification (launched 4/9/2026, decisions 4/10-4/30/2026), AD extract 05/15/2026, Netwrix revocations 4/16-4/24/2026</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -737,12 +734,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>In period - SAMPLE 1 (H2 2025)</t>
+          <t>SAMPLE 1 - covers Jul-Dec 2025</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>2025 Q3 SOX certification (launched 8/1/2025), AD extract 11/25/2025, Netwrix revocations</t>
+          <t>2025 Q3 SOX certification (launched 8/1/2025, decisions 8/6-8/28/2025), AD extract 11/25/2025, Netwrix revocations 9/2-9/8/2025</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -754,187 +751,19 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>03 Subsequent Period - Corroborative</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>2026 Q2 PAM BSI CyberArk Entitlement Owner Certification - Daily Active.csv</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Subsequent period - corroborative</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>2026 Q2 certification export (Jul-Sep 2026) - corroborative / IAMS identity status</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>2067</v>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>c256c8bb2d1028159e62837bde3f84d7</t>
-        </is>
-      </c>
-    </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>03 Subsequent Period - Corroborative</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>2026 Q2 PAM BSI CyberArk Manager Certification - Daily.csv</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Subsequent period - corroborative</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>2026 Q2 certification export (Jul-Sep 2026) - corroborative / IAMS identity status</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>356</v>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>9fb3dc4c9bc876618547eb3c9e83d827</t>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Only evidence within July 2025 - June 2026 is included. Files received 10/01/2026 outside the period (2025 Q1 and 2025 Q2 certifications - before; 2026 Q2 certification - after) are not relied on and are not in this folder.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>03 Subsequent Period - Corroborative</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>2026 Q2 PAM BSI SOX Entitlement Owner Certification - Daily Active.csv</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Subsequent period - corroborative</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>2026 Q2 certification export (Jul-Sep 2026) - corroborative / IAMS identity status</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="n">
-        <v>182</v>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>830c0819b2f629babf0e526644009451</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>03 Subsequent Period - Corroborative</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>2026 Q2 PAM BSI SOX Manager Certification - Validation1.csv</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Subsequent period - corroborative</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>2026 Q2 certification export (Jul-Sep 2026) - corroborative / IAMS identity status</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>78</v>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>51324252a99574321cc2f4722ad31bf7</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>03 Subsequent Period - Corroborative</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>BSI.IT.27.C7.02 Q2_2026.xlsx</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Subsequent period - corroborative</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>2026 Q2 tested workbook (launched 7/22/2026) - not counted as a sample</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="n">
-        <v>307</v>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>440e1675a4aff77304ff24eb4ac412cb</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n"/>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Not in this folder (kept in ..\BSI.IT.27.C7 New Testing Evidences-10-1--2026, as received 10/01/2026): BSI.IT.27.C7.02 Q1_2025 Cert.xlsx and 4 x 2025Q2 CSVs - prior period (before 07/2025), not relied on.</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Outstanding evidence: 2025 Q4 certification (A1 observation); management response / remediation plan for A5 and A6 exceptions.</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="n"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Outstanding: 2025 Q4 certification (A1 observation); management response / remediation plan for the A5 and A6 exceptions.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
BSI.IT.27.C7: restructure workpapers by the 9-step test procedure
- WP2 CPA: attribute table columns and summary of results organized by steps 1-9
- Walkthrough tab 2 grouped by steps 1-9; matrix headers mapped to steps
- Sample of 1 (2025 Q3, 2026 Q1): testing table by steps 1-9

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GtAt3iBzX5VYFEMTgXwPkP
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7 Network Device Admin Accoun/BSI.IT.27.C7 Final 07.2025-06.2026/BSI.IT.27.C7 Final Package Index.xlsx
+++ b/BSI.IT.27.C7 Network Device Admin Accoun/BSI.IT.27.C7 Final 07.2025-06.2026/BSI.IT.27.C7 Final Package Index.xlsx
@@ -534,11 +534,11 @@
         </is>
       </c>
       <c r="E6" s="3" t="n">
-        <v>2241</v>
+        <v>2242</v>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>0f92ac0c76c34ce2e95f6e992877927e</t>
+          <t>d69bc81c61e6a28be874845784875d6d</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>6efafa87d9b3e99793f1fb0387a42dea</t>
+          <t>865251c81f17f3343e939467d4d8f913</t>
         </is>
       </c>
     </row>
@@ -590,15 +590,15 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Step-by-step testing, attribute matrix A1-A7, item detail, exceptions (16 accounts), sources, evidence status, 9-step procedure coverage (tab 8)</t>
+          <t>Tab 2 step-by-step by the 9 test steps; attribute matrix; item detail; exceptions (16 accounts); sources; evidence status; tab 8 procedure coverage</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>04ee35dd7a05b191dd70b356e90f2565</t>
+          <t>a66a51632192f0981cfb26514e1a56a4</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Control Metadata, CDA, CPA (samples 2025 Q3 and 2026 Q1, rating Needs Improvement)</t>
+          <t>Control Metadata, CDA, CPA - test procedure and results by the 9 test steps; samples 2025 Q3 and 2026 Q1; rating Needs Improvement</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -628,7 +628,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>fdaebe5e247967ff82df95506aaf0b5d</t>
+          <t>bea02a9d5ae288e21a47303ad848df83</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BSI.IT.27.C7: add evidence request for the process owner
- BSI.IT.27.C7.06: 12 requests by test step, 16 account-level questions, path to pass

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GtAt3iBzX5VYFEMTgXwPkP
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7 Network Device Admin Accoun/BSI.IT.27.C7 Final 07.2025-06.2026/BSI.IT.27.C7 Final Package Index.xlsx
+++ b/BSI.IT.27.C7 Network Device Admin Accoun/BSI.IT.27.C7 Final 07.2025-06.2026/BSI.IT.27.C7 Final Package Index.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -635,30 +635,30 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>01 Policies and Procedures</t>
+          <t>00 Final Workpaper</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>BSI.IT.27.C7.01 Identity and Access Management Standard v10.0 09.29.2025.pdf</t>
+          <t>BSI.IT.27.C7.06 Evidence Request - Process Owner.xlsx</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Standard - in effect 09/29/2025 onward</t>
+          <t>Request to process owner</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>IAM Standard v10.0 - SUS.IAMS.4.2.5.19 privileged access at least semi-annually; 4.2.5.21 revocation within 30 business days</t>
+          <t>12 evidence requests (by test step), 16 account-level questions, path to pass per step</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>647</v>
+        <v>15</v>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>bc6cbef4c58ffd183348884d02a16cee</t>
+          <t>c51b2ef42507ea4ddc1078c04c1b66b5</t>
         </is>
       </c>
     </row>
@@ -670,25 +670,25 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>BSI.IT.27.C7.03 PAM Definition of Privilege.pdf</t>
+          <t>BSI.IT.27.C7.01 Identity and Access Management Standard v10.0 09.29.2025.pdf</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Policy - in effect whole period</t>
+          <t>Standard - in effect 09/29/2025 onward</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>PAM Definition of Privilege v10.0 (3/11/2025) sec. 3.3 - 4 privileged network AD groups</t>
+          <t>IAM Standard v10.0 - SUS.IAMS.4.2.5.19 privileged access at least semi-annually; 4.2.5.21 revocation within 30 business days</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>233</v>
+        <v>647</v>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>6e2cace9acada78339c9320ff92d9c7a</t>
+          <t>bc6cbef4c58ffd183348884d02a16cee</t>
         </is>
       </c>
     </row>
@@ -700,55 +700,55 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>PAM Recertification Procedure (BSI) 04.22.26.pdf</t>
+          <t>BSI.IT.27.C7.03 PAM Definition of Privilege.pdf</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Procedure - approved 04/22/2026</t>
+          <t>Policy - in effect whole period</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>PAM Recertification Procedure (BSI) v2.0 - control C7, quarterly SOX recertification, revocation (v1.0 of 04/22/2025 applied before)</t>
+          <t>PAM Definition of Privilege v10.0 (3/11/2025) sec. 3.3 - 4 privileged network AD groups</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>463</v>
+        <v>233</v>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>9eaef168c42e8bd6bdd088432f6bf75a</t>
+          <t>6e2cace9acada78339c9320ff92d9c7a</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>02 Evidence 07.2025-06.2026</t>
+          <t>01 Policies and Procedures</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>BSI.IT.27.C7.02 Q1 2026 Cert.xlsx</t>
+          <t>PAM Recertification Procedure (BSI) 04.22.26.pdf</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Evidence - SAMPLE 2 (Jan-Jun 2026)</t>
+          <t>Procedure - approved 04/22/2026</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>2026 Q1 SOX certification (launched 4/9/2026, decisions 4/10-4/30/2026), AD extract 05/15/2026, Netwrix revocations 4/16-4/24/2026</t>
+          <t>PAM Recertification Procedure (BSI) v2.0 - control C7, quarterly SOX recertification, revocation (v1.0 of 04/22/2025 applied before)</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>3063</v>
+        <v>463</v>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>8d338a2151c9c28eff23af70e6583695</t>
+          <t>9eaef168c42e8bd6bdd088432f6bf75a</t>
         </is>
       </c>
     </row>
@@ -760,38 +760,68 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
+          <t>BSI.IT.27.C7.02 Q1 2026 Cert.xlsx</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Evidence - SAMPLE 2 (Jan-Jun 2026)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>2026 Q1 SOX certification (launched 4/9/2026, decisions 4/10-4/30/2026), AD extract 05/15/2026, Netwrix revocations 4/16-4/24/2026</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>3063</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>8d338a2151c9c28eff23af70e6583695</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>02 Evidence 07.2025-06.2026</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
           <t>BSI.IT.27.C7.02 Q3_2025.xlsx</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Evidence - SAMPLE 1 (Jul-Dec 2025)</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>2025 Q3 SOX certification (launched 8/1/2025, decisions 8/6-8/28/2025), AD extract 11/25/2025, Netwrix revocations 9/2-9/8/2025</t>
         </is>
       </c>
-      <c r="E14" s="3" t="n">
+      <c r="E15" s="3" t="n">
         <v>3743</v>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>9df232d76e15d4e56a5f55da1d84aa4a</t>
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Only evidence within July 2025 - June 2026 is included. Out-of-period files received 10/01/2026 (2025 Q1 / 2025 Q2 certifications - before; 2026 Q2 certification and IAM Standard v11.0 of 07/28/2026 - after) are not relied on and are not in this folder.</t>
-        </is>
-      </c>
-    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
+        <is>
+          <t>Only evidence within July 2025 - June 2026 is included. Out-of-period files received 10/01/2026 (2025 Q1 / 2025 Q2 certifications - before; 2026 Q2 certification and IAM Standard v11.0 of 07/28/2026 - after) are not relied on and are not in this folder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Outstanding: 2025 Q4 certification (A1 observation); management response / remediation for A5 and A6; IAM Standard v9.0 and PAM Recertification Procedure v1.0 (versions in force at the 2025 Q3 review).</t>
         </is>

</xml_diff>